<commit_message>
feat: user can export RSPI as PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/RSPI Template.xlsx
+++ b/procurement_documents/RSPI Template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D90069-DC58-4AEA-A5E0-D858542FCF3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AF30D4-EF59-45BD-ADC2-927614EF1FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{FF649E56-644D-4834-98B7-02186BC6A766}"/>
   </bookViews>
@@ -552,50 +552,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -627,12 +585,6 @@
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -793,26 +745,68 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -822,12 +816,24 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -941,62 +947,6 @@
       <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="0" y="20193000"/>
-          <a:ext cx="438149" cy="457200"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>47626</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="438149" cy="457200"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{631A6E54-CC81-4ADF-BD40-1299A4464BB0}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="47626" y="57150"/>
           <a:ext cx="438149" cy="457200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1481,600 +1431,601 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B53CEC9-EC7F-473A-A392-BCE49FF1BF91}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:H187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="6.85546875" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="39.7109375" customWidth="1"/>
-    <col min="5" max="6" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="40.140625" customWidth="1"/>
+    <col min="5" max="6" width="5.5703125" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="80"/>
+    </row>
+    <row r="2" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="8"/>
-    </row>
-    <row r="3" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="84"/>
+    </row>
+    <row r="3" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="85" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="6" t="s">
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8"/>
-    </row>
-    <row r="4" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="84"/>
+    </row>
+    <row r="4" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="6" t="s">
+      <c r="B4" s="86"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="8"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
+      <c r="H4" s="84"/>
+    </row>
+    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="9" t="s">
+      <c r="B5" s="86"/>
+      <c r="C5" s="86"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="11"/>
-    </row>
-    <row r="6" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="14"/>
-    </row>
-    <row r="7" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="F5" s="86"/>
+      <c r="G5" s="86"/>
+      <c r="H5" s="87"/>
+    </row>
+    <row r="6" spans="1:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="88"/>
+      <c r="B6" s="89"/>
+      <c r="C6" s="89"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="90"/>
+    </row>
+    <row r="7" spans="1:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="20" t="s">
+      <c r="B8" s="5"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="21"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25" t="s">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="26"/>
-    </row>
-    <row r="10" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28" t="s">
+      <c r="B10" s="97"/>
+      <c r="C10" s="97"/>
+      <c r="D10" s="97"/>
+      <c r="E10" s="97"/>
+      <c r="F10" s="97"/>
+      <c r="G10" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="28"/>
-    </row>
-    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
+      <c r="H10" s="98"/>
+    </row>
+    <row r="11" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="29" t="s">
+      <c r="E11" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="29" t="s">
+      <c r="G11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="29" t="s">
+      <c r="H11" s="13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="46"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="50"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="46"/>
-      <c r="B17" s="47"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="46"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="53"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
-    </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="57"/>
-      <c r="B21" s="47"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="58"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="50"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="57"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="63"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="57"/>
-      <c r="B25" s="47"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="63"/>
-      <c r="B26" s="47"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="68"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="50"/>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="63"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="63"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="70"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="50"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="63"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="72"/>
-      <c r="E29" s="73"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="50"/>
-    </row>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="63"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="74"/>
-      <c r="E30" s="37"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="63"/>
-      <c r="B31" s="47"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="76"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="63"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="77"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="76"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="63"/>
-      <c r="B33" s="47"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="75"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
-    </row>
-    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="63"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="79"/>
-      <c r="D34" s="80"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="75"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="63"/>
-      <c r="B35" s="47"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="75"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="63"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="82"/>
-      <c r="E36" s="83"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="84"/>
-      <c r="H36" s="84"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="63"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="85"/>
-      <c r="E37" s="83"/>
-      <c r="F37" s="47"/>
-      <c r="G37" s="84"/>
-      <c r="H37" s="84"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="63"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="83"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="84"/>
-      <c r="H38" s="84"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="63"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="85"/>
-      <c r="E39" s="83"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="86"/>
-      <c r="H39" s="50">
+    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+    </row>
+    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="16"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+    </row>
+    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+    </row>
+    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="27"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+    </row>
+    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+    </row>
+    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+    </row>
+    <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="30"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+    </row>
+    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+    </row>
+    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+    </row>
+    <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="41"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+    </row>
+    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="16"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+    </row>
+    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="41"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="34"/>
+    </row>
+    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="47"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+    </row>
+    <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="41"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+    </row>
+    <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="47"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+    </row>
+    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="47"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
+    </row>
+    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="47"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+    </row>
+    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="47"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
+    </row>
+    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="47"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="58"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
+    </row>
+    <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="47"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="59"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="60"/>
+    </row>
+    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="47"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="60"/>
+    </row>
+    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="47"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="63"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
+    </row>
+    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="47"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="64"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="60"/>
+    </row>
+    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="47"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="63"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="60"/>
+    </row>
+    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="47"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="66"/>
+      <c r="E36" s="67"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+    </row>
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="47"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="69"/>
+      <c r="E37" s="67"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="68"/>
+      <c r="H37" s="68"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="47"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="69"/>
+      <c r="E38" s="67"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="68"/>
+      <c r="H38" s="68"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="47"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="67"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="70"/>
+      <c r="H39" s="34">
         <f>SUM(H12:H38)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="87" t="s">
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="101" t="s">
         <v>23</v>
       </c>
-      <c r="B40" s="87"/>
-      <c r="C40" s="87"/>
-      <c r="D40" s="87"/>
-      <c r="E40" s="88" t="s">
+      <c r="B40" s="102"/>
+      <c r="C40" s="102"/>
+      <c r="D40" s="103"/>
+      <c r="E40" s="99" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="88"/>
-      <c r="G40" s="88"/>
-      <c r="H40" s="88"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="89"/>
-      <c r="B41" s="89"/>
-      <c r="C41" s="89"/>
-      <c r="D41" s="89"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="89"/>
-      <c r="G41" s="89"/>
-      <c r="H41" s="89"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="89" t="s">
+      <c r="F40" s="99"/>
+      <c r="G40" s="99"/>
+      <c r="H40" s="99"/>
+    </row>
+    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="100"/>
+      <c r="B41" s="100"/>
+      <c r="C41" s="100"/>
+      <c r="D41" s="100"/>
+      <c r="E41" s="100"/>
+      <c r="F41" s="100"/>
+      <c r="G41" s="100"/>
+      <c r="H41" s="100"/>
+    </row>
+    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="89"/>
-      <c r="C42" s="89"/>
-      <c r="D42" s="89"/>
-      <c r="E42" s="89"/>
-      <c r="F42" s="89"/>
-      <c r="G42" s="89"/>
-      <c r="H42" s="89"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="90"/>
-      <c r="B43" s="91"/>
-      <c r="C43" s="91"/>
-      <c r="D43" s="92"/>
-      <c r="E43" s="93" t="s">
+      <c r="B42" s="100"/>
+      <c r="C42" s="100"/>
+      <c r="D42" s="100"/>
+      <c r="E42" s="100"/>
+      <c r="F42" s="100"/>
+      <c r="G42" s="100"/>
+      <c r="H42" s="100"/>
+    </row>
+    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="91"/>
+      <c r="B43" s="92"/>
+      <c r="C43" s="92"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="105" t="s">
         <v>26</v>
       </c>
-      <c r="F43" s="94"/>
-      <c r="G43" s="94"/>
-      <c r="H43" s="95" t="s">
+      <c r="F43" s="106"/>
+      <c r="G43" s="106"/>
+      <c r="H43" s="74" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="96"/>
-      <c r="B44" s="96"/>
-      <c r="C44" s="96"/>
-      <c r="D44" s="96"/>
-      <c r="E44" s="97" t="s">
+    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="94"/>
+      <c r="B44" s="94"/>
+      <c r="C44" s="94"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="F44" s="98"/>
-      <c r="G44" s="98"/>
-      <c r="H44" s="99" t="s">
+      <c r="F44" s="96"/>
+      <c r="G44" s="96"/>
+      <c r="H44" s="75" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="100"/>
-      <c r="B45" s="100"/>
-      <c r="C45" s="100"/>
-      <c r="D45" s="100"/>
-      <c r="E45" s="100"/>
-      <c r="F45" s="100"/>
-      <c r="G45" s="100"/>
-      <c r="H45" s="100"/>
+      <c r="A45" s="76"/>
+      <c r="B45" s="76"/>
+      <c r="C45" s="76"/>
+      <c r="D45" s="76"/>
+      <c r="E45" s="76"/>
+      <c r="F45" s="76"/>
+      <c r="G45" s="76"/>
+      <c r="H45" s="76"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="100"/>
-      <c r="B46" s="100"/>
-      <c r="C46" s="100"/>
-      <c r="D46" s="100"/>
-      <c r="E46" s="100"/>
-      <c r="F46" s="100"/>
-      <c r="G46" s="100"/>
-      <c r="H46" s="100"/>
+      <c r="A46" s="76"/>
+      <c r="B46" s="76"/>
+      <c r="C46" s="76"/>
+      <c r="D46" s="76"/>
+      <c r="E46" s="76"/>
+      <c r="F46" s="76"/>
+      <c r="G46" s="76"/>
+      <c r="H46" s="76"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="100"/>
-      <c r="B47" s="100"/>
-      <c r="C47" s="100"/>
-      <c r="D47" s="100"/>
-      <c r="E47" s="100"/>
-      <c r="F47" s="100"/>
-      <c r="G47" s="100"/>
-      <c r="H47" s="100"/>
+      <c r="A47" s="76"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="76"/>
+      <c r="D47" s="76"/>
+      <c r="E47" s="76"/>
+      <c r="F47" s="76"/>
+      <c r="G47" s="76"/>
+      <c r="H47" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="100"/>
-      <c r="B48" s="100"/>
-      <c r="C48" s="100"/>
-      <c r="D48" s="100"/>
-      <c r="E48" s="100"/>
-      <c r="F48" s="100"/>
-      <c r="G48" s="100"/>
-      <c r="H48" s="100"/>
+      <c r="A48" s="76"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="76"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="76"/>
+      <c r="F48" s="76"/>
+      <c r="G48" s="76"/>
+      <c r="H48" s="76"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="100"/>
-      <c r="B49" s="100"/>
-      <c r="C49" s="100"/>
-      <c r="D49" s="100"/>
-      <c r="E49" s="100"/>
-      <c r="F49" s="100"/>
-      <c r="G49" s="100"/>
-      <c r="H49" s="100"/>
+      <c r="A49" s="76"/>
+      <c r="B49" s="76"/>
+      <c r="C49" s="76"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="76"/>
+      <c r="F49" s="76"/>
+      <c r="G49" s="76"/>
+      <c r="H49" s="76"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="100"/>
-      <c r="B50" s="100"/>
-      <c r="C50" s="100"/>
-      <c r="D50" s="100"/>
-      <c r="E50" s="100"/>
-      <c r="F50" s="100"/>
-      <c r="G50" s="100"/>
-      <c r="H50" s="100"/>
+      <c r="A50" s="76"/>
+      <c r="B50" s="76"/>
+      <c r="C50" s="76"/>
+      <c r="D50" s="76"/>
+      <c r="E50" s="76"/>
+      <c r="F50" s="76"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="76"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="100"/>
-      <c r="B51" s="100"/>
-      <c r="C51" s="100"/>
-      <c r="D51" s="100"/>
-      <c r="E51" s="100"/>
-      <c r="F51" s="100"/>
-      <c r="G51" s="100"/>
-      <c r="H51" s="100"/>
+      <c r="A51" s="76"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="76"/>
+      <c r="D51" s="76"/>
+      <c r="E51" s="76"/>
+      <c r="F51" s="76"/>
+      <c r="G51" s="76"/>
+      <c r="H51" s="76"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="100"/>
-      <c r="B52" s="100"/>
-      <c r="C52" s="100"/>
-      <c r="D52" s="100"/>
-      <c r="E52" s="100"/>
-      <c r="F52" s="100"/>
-      <c r="G52" s="100"/>
-      <c r="H52" s="100"/>
+      <c r="A52" s="76"/>
+      <c r="B52" s="76"/>
+      <c r="C52" s="76"/>
+      <c r="D52" s="76"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="76"/>
+      <c r="G52" s="76"/>
+      <c r="H52" s="76"/>
     </row>
     <row r="62" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="113" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2083,7 +2034,7 @@
     <row r="180" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="187" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="24">
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="E44:G44"/>
@@ -2094,6 +2045,8 @@
     <mergeCell ref="E41:H41"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="E42:H42"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E43:G43"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="A5:D5"/>
@@ -2116,6 +2069,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60B6E1F8-2B35-4BED-B4EF-E9B2A4393D42}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2129,615 +2083,615 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="80"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="8"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="84"/>
     </row>
     <row r="3" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="85" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="6" t="s">
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="84"/>
     </row>
     <row r="4" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="6" t="s">
+      <c r="B4" s="86"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="8"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
+      <c r="H4" s="84"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="9" t="s">
+      <c r="B5" s="86"/>
+      <c r="C5" s="86"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="11"/>
+      <c r="F5" s="86"/>
+      <c r="G5" s="86"/>
+      <c r="H5" s="87"/>
     </row>
     <row r="6" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="14"/>
+      <c r="A6" s="88"/>
+      <c r="B6" s="89"/>
+      <c r="C6" s="89"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="88"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="90"/>
     </row>
     <row r="7" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="20" t="s">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="26" t="s">
+      <c r="H9" s="12" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="97" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28" t="s">
+      <c r="B10" s="97"/>
+      <c r="C10" s="97"/>
+      <c r="D10" s="97"/>
+      <c r="E10" s="97"/>
+      <c r="F10" s="97"/>
+      <c r="G10" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="28"/>
+      <c r="H10" s="98"/>
     </row>
     <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="29" t="s">
+      <c r="E11" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="29" t="s">
+      <c r="G11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="29" t="s">
+      <c r="H11" s="13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="E12" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="38" t="s">
+      <c r="G12" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="38" t="s">
+      <c r="H12" s="22" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="46"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="50"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="46"/>
-      <c r="B17" s="47"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="46"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="53"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
+      <c r="A18" s="30"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="57"/>
-      <c r="B21" s="47"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="58"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
+      <c r="A21" s="41"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="50"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="57"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
+      <c r="A23" s="41"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="34"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="63"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
+      <c r="A24" s="47"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="57"/>
-      <c r="B25" s="47"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
+      <c r="A25" s="41"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="63"/>
-      <c r="B26" s="47"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="68"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="50"/>
+      <c r="A26" s="47"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="63"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
+      <c r="A27" s="47"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="63"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="70"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="50"/>
+      <c r="A28" s="47"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="63"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="72"/>
-      <c r="E29" s="73"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="50"/>
+      <c r="A29" s="47"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="63"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="74"/>
-      <c r="E30" s="37"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
+      <c r="A30" s="47"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="58"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="63"/>
-      <c r="B31" s="47"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="76"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="59"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="60"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="63"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="77"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="76"/>
+      <c r="A32" s="47"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="60"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="63"/>
-      <c r="B33" s="47"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="75"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="A33" s="47"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="63"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
     </row>
     <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="63"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="79"/>
-      <c r="D34" s="80"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="75"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="A34" s="47"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="64"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="60"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="63"/>
-      <c r="B35" s="47"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="75"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="A35" s="47"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="63"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="60"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="63"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="82"/>
-      <c r="E36" s="83"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="84"/>
-      <c r="H36" s="84"/>
+      <c r="A36" s="47"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="66"/>
+      <c r="E36" s="67"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="63"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="85"/>
-      <c r="E37" s="83"/>
-      <c r="F37" s="47"/>
-      <c r="G37" s="84"/>
-      <c r="H37" s="84"/>
+      <c r="A37" s="47"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="69"/>
+      <c r="E37" s="67"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="68"/>
+      <c r="H37" s="68"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="63"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="83"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="84"/>
-      <c r="H38" s="84"/>
+      <c r="A38" s="47"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="69"/>
+      <c r="E38" s="67"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="68"/>
+      <c r="H38" s="68"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="63"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="85"/>
-      <c r="E39" s="83"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="86"/>
-      <c r="H39" s="50">
+      <c r="A39" s="47"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="67"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="70"/>
+      <c r="H39" s="34">
         <f>SUM(H12:H38)</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="87" t="s">
+      <c r="A40" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="B40" s="87"/>
-      <c r="C40" s="87"/>
-      <c r="D40" s="87"/>
-      <c r="E40" s="88" t="s">
+      <c r="B40" s="71"/>
+      <c r="C40" s="71"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="99" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="88"/>
-      <c r="G40" s="88"/>
-      <c r="H40" s="88"/>
+      <c r="F40" s="99"/>
+      <c r="G40" s="99"/>
+      <c r="H40" s="99"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="89"/>
-      <c r="B41" s="89"/>
-      <c r="C41" s="89"/>
-      <c r="D41" s="89"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="89"/>
-      <c r="G41" s="89"/>
-      <c r="H41" s="89"/>
+      <c r="A41" s="100"/>
+      <c r="B41" s="100"/>
+      <c r="C41" s="100"/>
+      <c r="D41" s="100"/>
+      <c r="E41" s="100"/>
+      <c r="F41" s="100"/>
+      <c r="G41" s="100"/>
+      <c r="H41" s="100"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="89" t="s">
+      <c r="A42" s="100" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="89"/>
-      <c r="C42" s="89"/>
-      <c r="D42" s="89"/>
-      <c r="E42" s="89"/>
-      <c r="F42" s="89"/>
-      <c r="G42" s="89"/>
-      <c r="H42" s="89"/>
+      <c r="B42" s="100"/>
+      <c r="C42" s="100"/>
+      <c r="D42" s="100"/>
+      <c r="E42" s="100"/>
+      <c r="F42" s="100"/>
+      <c r="G42" s="100"/>
+      <c r="H42" s="100"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="90" t="s">
+      <c r="A43" s="91" t="s">
         <v>34</v>
       </c>
-      <c r="B43" s="91"/>
-      <c r="C43" s="91"/>
-      <c r="D43" s="92"/>
-      <c r="E43" s="93" t="s">
+      <c r="B43" s="92"/>
+      <c r="C43" s="92"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="F43" s="94"/>
-      <c r="G43" s="94"/>
-      <c r="H43" s="95" t="s">
+      <c r="F43" s="73"/>
+      <c r="G43" s="73"/>
+      <c r="H43" s="74" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="96" t="s">
+      <c r="A44" s="94" t="s">
         <v>35</v>
       </c>
-      <c r="B44" s="96"/>
-      <c r="C44" s="96"/>
-      <c r="D44" s="96"/>
-      <c r="E44" s="97" t="s">
+      <c r="B44" s="94"/>
+      <c r="C44" s="94"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="F44" s="98"/>
-      <c r="G44" s="98"/>
-      <c r="H44" s="99" t="s">
+      <c r="F44" s="96"/>
+      <c r="G44" s="96"/>
+      <c r="H44" s="75" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="100"/>
-      <c r="B45" s="100"/>
-      <c r="C45" s="100"/>
-      <c r="D45" s="100"/>
-      <c r="E45" s="100"/>
-      <c r="F45" s="100"/>
-      <c r="G45" s="100"/>
-      <c r="H45" s="100"/>
+      <c r="A45" s="76"/>
+      <c r="B45" s="76"/>
+      <c r="C45" s="76"/>
+      <c r="D45" s="76"/>
+      <c r="E45" s="76"/>
+      <c r="F45" s="76"/>
+      <c r="G45" s="76"/>
+      <c r="H45" s="76"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="100"/>
-      <c r="B46" s="100"/>
-      <c r="C46" s="100"/>
-      <c r="D46" s="100"/>
-      <c r="E46" s="100"/>
-      <c r="F46" s="100"/>
-      <c r="G46" s="100"/>
-      <c r="H46" s="100"/>
+      <c r="A46" s="76"/>
+      <c r="B46" s="76"/>
+      <c r="C46" s="76"/>
+      <c r="D46" s="76"/>
+      <c r="E46" s="76"/>
+      <c r="F46" s="76"/>
+      <c r="G46" s="76"/>
+      <c r="H46" s="76"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="100"/>
-      <c r="B47" s="100"/>
-      <c r="C47" s="100"/>
-      <c r="D47" s="100"/>
-      <c r="E47" s="100"/>
-      <c r="F47" s="100"/>
-      <c r="G47" s="100"/>
-      <c r="H47" s="100"/>
+      <c r="A47" s="76"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="76"/>
+      <c r="D47" s="76"/>
+      <c r="E47" s="76"/>
+      <c r="F47" s="76"/>
+      <c r="G47" s="76"/>
+      <c r="H47" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="100"/>
-      <c r="B48" s="100"/>
-      <c r="C48" s="100"/>
-      <c r="D48" s="100"/>
-      <c r="E48" s="100"/>
-      <c r="F48" s="100"/>
-      <c r="G48" s="100"/>
-      <c r="H48" s="100"/>
+      <c r="A48" s="76"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="76"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="76"/>
+      <c r="F48" s="76"/>
+      <c r="G48" s="76"/>
+      <c r="H48" s="76"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="100"/>
-      <c r="B49" s="100"/>
-      <c r="C49" s="100"/>
-      <c r="D49" s="100"/>
-      <c r="E49" s="100"/>
-      <c r="F49" s="100"/>
-      <c r="G49" s="100"/>
-      <c r="H49" s="100"/>
+      <c r="A49" s="76"/>
+      <c r="B49" s="76"/>
+      <c r="C49" s="76"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="76"/>
+      <c r="F49" s="76"/>
+      <c r="G49" s="76"/>
+      <c r="H49" s="76"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="100"/>
-      <c r="B50" s="100"/>
-      <c r="C50" s="100"/>
-      <c r="D50" s="100"/>
-      <c r="E50" s="100"/>
-      <c r="F50" s="100"/>
-      <c r="G50" s="100"/>
-      <c r="H50" s="100"/>
+      <c r="A50" s="76"/>
+      <c r="B50" s="76"/>
+      <c r="C50" s="76"/>
+      <c r="D50" s="76"/>
+      <c r="E50" s="76"/>
+      <c r="F50" s="76"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="76"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="100"/>
-      <c r="B51" s="100"/>
-      <c r="C51" s="100"/>
-      <c r="D51" s="100"/>
-      <c r="E51" s="100"/>
-      <c r="F51" s="100"/>
-      <c r="G51" s="100"/>
-      <c r="H51" s="100"/>
+      <c r="A51" s="76"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="76"/>
+      <c r="D51" s="76"/>
+      <c r="E51" s="76"/>
+      <c r="F51" s="76"/>
+      <c r="G51" s="76"/>
+      <c r="H51" s="76"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="100"/>
-      <c r="B52" s="100"/>
-      <c r="C52" s="100"/>
-      <c r="D52" s="100"/>
-      <c r="E52" s="100"/>
-      <c r="F52" s="100"/>
-      <c r="G52" s="100"/>
-      <c r="H52" s="100"/>
+      <c r="A52" s="76"/>
+      <c r="B52" s="76"/>
+      <c r="C52" s="76"/>
+      <c r="D52" s="76"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="76"/>
+      <c r="G52" s="76"/>
+      <c r="H52" s="76"/>
     </row>
     <row r="62" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="113" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
chore: add tup logo in RSPI pdf
</commit_message>
<xml_diff>
--- a/procurement_documents/RSPI Template.xlsx
+++ b/procurement_documents/RSPI Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AF30D4-EF59-45BD-ADC2-927614EF1FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E875CDC2-2E5C-492D-B29A-110B8A9012C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{FF649E56-644D-4834-98B7-02186BC6A766}"/>
   </bookViews>
@@ -45,8 +45,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -178,6 +200,10 @@
   </si>
   <si>
     <t>rspi_amount</t>
+  </si>
+  <si>
+    <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES
+                                TAGUIG CITY</t>
   </si>
 </sst>
 </file>
@@ -552,7 +578,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -756,48 +782,10 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -831,9 +819,101 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1168,6 +1248,70 @@
 </externalLink>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1439,88 +1583,89 @@
     <col min="2" max="2" width="6.85546875" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="4" width="40.140625" customWidth="1"/>
-    <col min="5" max="6" width="5.5703125" customWidth="1"/>
+    <col min="5" max="5" width="7.28515625" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="80"/>
+      <c r="A1" s="104" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B1" s="113" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="109"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="106"/>
     </row>
     <row r="2" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="81" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="82" t="s">
+      <c r="A2" s="108"/>
+      <c r="B2" s="111"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="97" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="99"/>
     </row>
     <row r="3" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="86"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="82" t="s">
+      <c r="B3" s="114"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="84"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="99"/>
     </row>
     <row r="4" spans="1:8" ht="24.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="86"/>
-      <c r="C4" s="86"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="82" t="s">
+      <c r="B4" s="114"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="96"/>
+      <c r="E4" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="84"/>
+      <c r="F4" s="98"/>
+      <c r="G4" s="98"/>
+      <c r="H4" s="99"/>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="85" t="s">
+      <c r="A5" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="86"/>
-      <c r="C5" s="86"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="85" t="s">
+      <c r="B5" s="114"/>
+      <c r="C5" s="114"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="86"/>
-      <c r="G5" s="86"/>
-      <c r="H5" s="87"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="95"/>
+      <c r="H5" s="96"/>
     </row>
     <row r="6" spans="1:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="88"/>
-      <c r="B6" s="89"/>
-      <c r="C6" s="89"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89"/>
-      <c r="G6" s="89"/>
-      <c r="H6" s="90"/>
+      <c r="A6" s="100"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="100"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="102"/>
     </row>
     <row r="7" spans="1:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1533,7 +1678,7 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="104" t="s">
+      <c r="A8" s="78" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="5"/>
@@ -1561,18 +1706,18 @@
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="97" t="s">
+      <c r="A10" s="85" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="97"/>
-      <c r="C10" s="97"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="97"/>
-      <c r="F10" s="97"/>
-      <c r="G10" s="98" t="s">
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="98"/>
+      <c r="H10" s="86"/>
     </row>
     <row r="11" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
@@ -1601,39 +1746,39 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="18"/>
+      <c r="A12" s="118"/>
+      <c r="B12" s="115"/>
+      <c r="C12" s="50"/>
       <c r="D12" s="19"/>
       <c r="E12" s="20"/>
-      <c r="F12" s="21"/>
+      <c r="F12" s="52"/>
       <c r="G12" s="22"/>
       <c r="H12" s="22"/>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="18"/>
+      <c r="A13" s="118"/>
+      <c r="B13" s="116"/>
+      <c r="C13" s="50"/>
       <c r="D13" s="24"/>
       <c r="E13" s="20"/>
-      <c r="F13" s="21"/>
+      <c r="F13" s="52"/>
       <c r="G13" s="22"/>
       <c r="H13" s="22"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="25"/>
+      <c r="A14" s="118"/>
+      <c r="B14" s="115"/>
+      <c r="C14" s="122"/>
       <c r="D14" s="19"/>
       <c r="E14" s="20"/>
-      <c r="F14" s="26"/>
+      <c r="F14" s="123"/>
       <c r="G14" s="22"/>
       <c r="H14" s="22"/>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="18"/>
+      <c r="A15" s="119"/>
+      <c r="B15" s="115"/>
+      <c r="C15" s="50"/>
       <c r="D15" s="28"/>
       <c r="E15" s="20"/>
       <c r="F15" s="29"/>
@@ -1641,9 +1786,9 @@
       <c r="H15" s="22"/>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="30"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="18"/>
+      <c r="A16" s="120"/>
+      <c r="B16" s="117"/>
+      <c r="C16" s="50"/>
       <c r="D16" s="32"/>
       <c r="E16" s="33"/>
       <c r="F16" s="29"/>
@@ -1651,9 +1796,9 @@
       <c r="H16" s="34"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="18"/>
+      <c r="A17" s="120"/>
+      <c r="B17" s="117"/>
+      <c r="C17" s="50"/>
       <c r="D17" s="28"/>
       <c r="E17" s="21"/>
       <c r="F17" s="29"/>
@@ -1661,9 +1806,9 @@
       <c r="H17" s="34"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
+      <c r="A18" s="120"/>
+      <c r="B18" s="115"/>
+      <c r="C18" s="50"/>
       <c r="D18" s="35"/>
       <c r="E18" s="36"/>
       <c r="F18" s="37"/>
@@ -1671,29 +1816,29 @@
       <c r="H18" s="34"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
+      <c r="A19" s="118"/>
+      <c r="B19" s="115"/>
+      <c r="C19" s="50"/>
       <c r="D19" s="35"/>
       <c r="E19" s="33"/>
-      <c r="F19" s="38"/>
+      <c r="F19" s="124"/>
       <c r="G19" s="34"/>
       <c r="H19" s="34"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="18"/>
+      <c r="A20" s="118"/>
+      <c r="B20" s="115"/>
+      <c r="C20" s="50"/>
       <c r="D20" s="32"/>
       <c r="E20" s="39"/>
-      <c r="F20" s="38"/>
+      <c r="F20" s="124"/>
       <c r="G20" s="40"/>
       <c r="H20" s="40"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="41"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="18"/>
+      <c r="A21" s="121"/>
+      <c r="B21" s="117"/>
+      <c r="C21" s="50"/>
       <c r="D21" s="19"/>
       <c r="E21" s="42"/>
       <c r="F21" s="43"/>
@@ -1701,48 +1846,48 @@
       <c r="H21" s="40"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
+      <c r="A22" s="118"/>
+      <c r="B22" s="115"/>
+      <c r="C22" s="50"/>
       <c r="D22" s="44"/>
       <c r="E22" s="33"/>
-      <c r="F22" s="21"/>
+      <c r="F22" s="52"/>
       <c r="G22" s="34"/>
       <c r="H22" s="34"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="41"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="18"/>
+      <c r="A23" s="121"/>
+      <c r="B23" s="117"/>
+      <c r="C23" s="50"/>
       <c r="D23" s="45"/>
       <c r="E23" s="46"/>
-      <c r="F23" s="21"/>
+      <c r="F23" s="52"/>
       <c r="G23" s="34"/>
       <c r="H23" s="34"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="47"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="18"/>
+      <c r="A24" s="115"/>
+      <c r="B24" s="117"/>
+      <c r="C24" s="50"/>
       <c r="D24" s="48"/>
       <c r="E24" s="46"/>
-      <c r="F24" s="21"/>
+      <c r="F24" s="52"/>
       <c r="G24" s="34"/>
       <c r="H24" s="34"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="41"/>
-      <c r="B25" s="31"/>
-      <c r="C25" s="18"/>
+      <c r="A25" s="121"/>
+      <c r="B25" s="117"/>
+      <c r="C25" s="50"/>
       <c r="D25" s="49"/>
       <c r="E25" s="46"/>
-      <c r="F25" s="21"/>
+      <c r="F25" s="52"/>
       <c r="G25" s="34"/>
       <c r="H25" s="34"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="47"/>
-      <c r="B26" s="31"/>
+      <c r="A26" s="115"/>
+      <c r="B26" s="117"/>
       <c r="C26" s="50"/>
       <c r="D26" s="51"/>
       <c r="E26" s="46"/>
@@ -1751,49 +1896,49 @@
       <c r="H26" s="34"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="47"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="18"/>
+      <c r="A27" s="115"/>
+      <c r="B27" s="117"/>
+      <c r="C27" s="50"/>
       <c r="D27" s="53"/>
       <c r="E27" s="46"/>
-      <c r="F27" s="21"/>
+      <c r="F27" s="52"/>
       <c r="G27" s="34"/>
       <c r="H27" s="34"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="47"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="18"/>
+      <c r="A28" s="115"/>
+      <c r="B28" s="117"/>
+      <c r="C28" s="50"/>
       <c r="D28" s="54"/>
       <c r="E28" s="55"/>
-      <c r="F28" s="21"/>
+      <c r="F28" s="52"/>
       <c r="G28" s="34"/>
       <c r="H28" s="34"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="47"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="18"/>
+      <c r="A29" s="115"/>
+      <c r="B29" s="117"/>
+      <c r="C29" s="50"/>
       <c r="D29" s="56"/>
       <c r="E29" s="57"/>
-      <c r="F29" s="21"/>
+      <c r="F29" s="52"/>
       <c r="G29" s="34"/>
       <c r="H29" s="34"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="47"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="18"/>
+      <c r="A30" s="115"/>
+      <c r="B30" s="117"/>
+      <c r="C30" s="50"/>
       <c r="D30" s="58"/>
       <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
+      <c r="F30" s="52"/>
       <c r="G30" s="34"/>
       <c r="H30" s="34"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="47"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="18"/>
+      <c r="A31" s="115"/>
+      <c r="B31" s="117"/>
+      <c r="C31" s="50"/>
       <c r="D31" s="54"/>
       <c r="E31" s="21"/>
       <c r="F31" s="59"/>
@@ -1801,9 +1946,9 @@
       <c r="H31" s="60"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="47"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="18"/>
+      <c r="A32" s="115"/>
+      <c r="B32" s="117"/>
+      <c r="C32" s="50"/>
       <c r="D32" s="61"/>
       <c r="E32" s="62"/>
       <c r="F32" s="59"/>
@@ -1811,9 +1956,9 @@
       <c r="H32" s="60"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="47"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="63"/>
+      <c r="A33" s="115"/>
+      <c r="B33" s="117"/>
+      <c r="C33" s="77"/>
       <c r="D33" s="64"/>
       <c r="E33" s="65"/>
       <c r="F33" s="59"/>
@@ -1821,9 +1966,9 @@
       <c r="H33" s="60"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="47"/>
-      <c r="B34" s="31"/>
-      <c r="C34" s="63"/>
+      <c r="A34" s="115"/>
+      <c r="B34" s="117"/>
+      <c r="C34" s="77"/>
       <c r="D34" s="64"/>
       <c r="E34" s="65"/>
       <c r="F34" s="59"/>
@@ -1831,9 +1976,9 @@
       <c r="H34" s="60"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="47"/>
-      <c r="B35" s="31"/>
-      <c r="C35" s="63"/>
+      <c r="A35" s="115"/>
+      <c r="B35" s="117"/>
+      <c r="C35" s="77"/>
       <c r="D35" s="48"/>
       <c r="E35" s="65"/>
       <c r="F35" s="59"/>
@@ -1841,42 +1986,42 @@
       <c r="H35" s="60"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="47"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
+      <c r="A36" s="115"/>
+      <c r="B36" s="117"/>
+      <c r="C36" s="117"/>
       <c r="D36" s="66"/>
       <c r="E36" s="67"/>
-      <c r="F36" s="31"/>
+      <c r="F36" s="117"/>
       <c r="G36" s="68"/>
       <c r="H36" s="68"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="47"/>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
+      <c r="A37" s="115"/>
+      <c r="B37" s="117"/>
+      <c r="C37" s="117"/>
       <c r="D37" s="69"/>
       <c r="E37" s="67"/>
-      <c r="F37" s="31"/>
+      <c r="F37" s="117"/>
       <c r="G37" s="68"/>
       <c r="H37" s="68"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="47"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
+      <c r="A38" s="115"/>
+      <c r="B38" s="117"/>
+      <c r="C38" s="117"/>
       <c r="D38" s="69"/>
       <c r="E38" s="67"/>
-      <c r="F38" s="31"/>
+      <c r="F38" s="117"/>
       <c r="G38" s="68"/>
       <c r="H38" s="68"/>
     </row>
     <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="47"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
+      <c r="A39" s="115"/>
+      <c r="B39" s="117"/>
+      <c r="C39" s="117"/>
       <c r="D39" s="69"/>
       <c r="E39" s="67"/>
-      <c r="F39" s="31"/>
+      <c r="F39" s="117"/>
       <c r="G39" s="70"/>
       <c r="H39" s="34">
         <f>SUM(H12:H38)</f>
@@ -1884,65 +2029,65 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="101" t="s">
+      <c r="A40" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="B40" s="102"/>
-      <c r="C40" s="102"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="99" t="s">
+      <c r="B40" s="90"/>
+      <c r="C40" s="90"/>
+      <c r="D40" s="91"/>
+      <c r="E40" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="99"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="99"/>
+      <c r="F40" s="87"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="87"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="100"/>
-      <c r="B41" s="100"/>
-      <c r="C41" s="100"/>
-      <c r="D41" s="100"/>
-      <c r="E41" s="100"/>
-      <c r="F41" s="100"/>
-      <c r="G41" s="100"/>
-      <c r="H41" s="100"/>
+      <c r="A41" s="88"/>
+      <c r="B41" s="88"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="88"/>
+      <c r="E41" s="88"/>
+      <c r="F41" s="88"/>
+      <c r="G41" s="88"/>
+      <c r="H41" s="88"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="100" t="s">
+      <c r="A42" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="100"/>
-      <c r="C42" s="100"/>
-      <c r="D42" s="100"/>
-      <c r="E42" s="100"/>
-      <c r="F42" s="100"/>
-      <c r="G42" s="100"/>
-      <c r="H42" s="100"/>
+      <c r="B42" s="88"/>
+      <c r="C42" s="88"/>
+      <c r="D42" s="88"/>
+      <c r="E42" s="88"/>
+      <c r="F42" s="88"/>
+      <c r="G42" s="88"/>
+      <c r="H42" s="88"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="91"/>
-      <c r="B43" s="92"/>
-      <c r="C43" s="92"/>
-      <c r="D43" s="93"/>
-      <c r="E43" s="105" t="s">
+      <c r="A43" s="79"/>
+      <c r="B43" s="80"/>
+      <c r="C43" s="80"/>
+      <c r="D43" s="81"/>
+      <c r="E43" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="F43" s="106"/>
-      <c r="G43" s="106"/>
+      <c r="F43" s="93"/>
+      <c r="G43" s="93"/>
       <c r="H43" s="74" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="94"/>
-      <c r="B44" s="94"/>
-      <c r="C44" s="94"/>
-      <c r="D44" s="94"/>
-      <c r="E44" s="95" t="s">
+      <c r="A44" s="82"/>
+      <c r="B44" s="82"/>
+      <c r="C44" s="82"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="F44" s="96"/>
-      <c r="G44" s="96"/>
+      <c r="F44" s="84"/>
+      <c r="G44" s="84"/>
       <c r="H44" s="75" t="s">
         <v>29</v>
       </c>
@@ -2035,6 +2180,18 @@
     <row r="187" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="E44:G44"/>
@@ -2047,18 +2204,6 @@
     <mergeCell ref="E42:H42"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="E43:G43"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.98425196850393704" bottom="0.23622047244094499" header="3.9370078740157501E-2" footer="3.9370078740157501E-2"/>
@@ -2083,82 +2228,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="80"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="106"/>
     </row>
     <row r="2" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="81" t="s">
+      <c r="A2" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="82" t="s">
+      <c r="B2" s="107"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="97" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="99"/>
     </row>
     <row r="3" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="86"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="82" t="s">
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="84"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="99"/>
     </row>
     <row r="4" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="86"/>
-      <c r="C4" s="86"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="82" t="s">
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="96"/>
+      <c r="E4" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="84"/>
+      <c r="F4" s="98"/>
+      <c r="G4" s="98"/>
+      <c r="H4" s="99"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="85" t="s">
+      <c r="A5" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="86"/>
-      <c r="C5" s="86"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="85" t="s">
+      <c r="B5" s="95"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="86"/>
-      <c r="G5" s="86"/>
-      <c r="H5" s="87"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="95"/>
+      <c r="H5" s="96"/>
     </row>
     <row r="6" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="88"/>
-      <c r="B6" s="89"/>
-      <c r="C6" s="89"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89"/>
-      <c r="G6" s="89"/>
-      <c r="H6" s="90"/>
+      <c r="A6" s="100"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="100"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="102"/>
     </row>
     <row r="7" spans="1:8" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2207,18 +2352,18 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="97" t="s">
+      <c r="A10" s="85" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="97"/>
-      <c r="C10" s="97"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="97"/>
-      <c r="F10" s="97"/>
-      <c r="G10" s="98" t="s">
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="98"/>
+      <c r="H10" s="86"/>
     </row>
     <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
@@ -2552,42 +2697,42 @@
       <c r="B40" s="71"/>
       <c r="C40" s="71"/>
       <c r="D40" s="71"/>
-      <c r="E40" s="99" t="s">
+      <c r="E40" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="99"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="99"/>
+      <c r="F40" s="87"/>
+      <c r="G40" s="87"/>
+      <c r="H40" s="87"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="100"/>
-      <c r="B41" s="100"/>
-      <c r="C41" s="100"/>
-      <c r="D41" s="100"/>
-      <c r="E41" s="100"/>
-      <c r="F41" s="100"/>
-      <c r="G41" s="100"/>
-      <c r="H41" s="100"/>
+      <c r="A41" s="88"/>
+      <c r="B41" s="88"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="88"/>
+      <c r="E41" s="88"/>
+      <c r="F41" s="88"/>
+      <c r="G41" s="88"/>
+      <c r="H41" s="88"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="100" t="s">
+      <c r="A42" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="B42" s="100"/>
-      <c r="C42" s="100"/>
-      <c r="D42" s="100"/>
-      <c r="E42" s="100"/>
-      <c r="F42" s="100"/>
-      <c r="G42" s="100"/>
-      <c r="H42" s="100"/>
+      <c r="B42" s="88"/>
+      <c r="C42" s="88"/>
+      <c r="D42" s="88"/>
+      <c r="E42" s="88"/>
+      <c r="F42" s="88"/>
+      <c r="G42" s="88"/>
+      <c r="H42" s="88"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="91" t="s">
+      <c r="A43" s="79" t="s">
         <v>34</v>
       </c>
-      <c r="B43" s="92"/>
-      <c r="C43" s="92"/>
-      <c r="D43" s="93"/>
+      <c r="B43" s="80"/>
+      <c r="C43" s="80"/>
+      <c r="D43" s="81"/>
       <c r="E43" s="72" t="s">
         <v>26</v>
       </c>
@@ -2598,17 +2743,17 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="94" t="s">
+      <c r="A44" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="B44" s="94"/>
-      <c r="C44" s="94"/>
-      <c r="D44" s="94"/>
-      <c r="E44" s="95" t="s">
+      <c r="B44" s="82"/>
+      <c r="C44" s="82"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="F44" s="96"/>
-      <c r="G44" s="96"/>
+      <c r="F44" s="84"/>
+      <c r="G44" s="84"/>
       <c r="H44" s="75" t="s">
         <v>29</v>
       </c>
@@ -2701,6 +2846,18 @@
     <row r="187" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="E44:G44"/>
@@ -2711,18 +2868,6 @@
     <mergeCell ref="E41:H41"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="E42:H42"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.98425196850393704" bottom="0.23622047244094499" header="3.9370078740157501E-2" footer="3.9370078740157501E-2"/>

</xml_diff>